<commit_message>
feat(gp-026): complete Kimball star-schema, tableau LOD calculations and executive excel scorecard
</commit_message>
<xml_diff>
--- a/reports/Executive_Hiring_Scorecard.xlsx
+++ b/reports/Executive_Hiring_Scorecard.xlsx
@@ -137,11 +137,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -517,7 +517,7 @@
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="29" customWidth="1" min="7" max="7"/>
   </cols>
@@ -570,27 +570,27 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>1,916</t>
+          <t>2,377</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>3.83%</t>
+          <t>4.75%</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>8.8 Days</t>
+          <t>22.1 Days</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>$53,704,410</t>
+          <t>$87,111,395</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>$28,029</t>
+          <t>$36,648</t>
         </is>
       </c>
     </row>
@@ -643,18 +643,18 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>1_Applied</t>
+          <t>1_Application_Review</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>30663</v>
+        <v>20302</v>
       </c>
       <c r="C9" s="8" t="n">
-        <v>0.6133</v>
+        <v>0.406</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>2.5 Days</t>
+          <t>14.0 Days</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
@@ -671,18 +671,18 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>2_Screening_Passed</t>
+          <t>2_Technical_Screening</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>9689</v>
+        <v>12686</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>0.1938</v>
+        <v>0.2537</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>9.5 Days</t>
+          <t>21.0 Days</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
@@ -699,18 +699,18 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>3_Technical_Passed</t>
+          <t>3_System_Design_Interview</t>
         </is>
       </c>
       <c r="B11" s="7" t="n">
-        <v>4969</v>
+        <v>9113</v>
       </c>
       <c r="C11" s="8" t="n">
-        <v>0.09939999999999999</v>
+        <v>0.1823</v>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>19.6 Days</t>
+          <t>28.0 Days</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr">
@@ -727,18 +727,18 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>4_Executive_Passed</t>
+          <t>4_Cultural_Fit</t>
         </is>
       </c>
       <c r="B12" s="7" t="n">
-        <v>2763</v>
+        <v>4752</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>0.0553</v>
+        <v>0.095</v>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>31.5 Days</t>
+          <t>35.0 Days</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
@@ -755,35 +755,35 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>5_Offer_Accepted</t>
+          <t>5_Executive_Offer</t>
         </is>
       </c>
       <c r="B13" s="7" t="n">
-        <v>1916</v>
+        <v>3147</v>
       </c>
       <c r="C13" s="8" t="n">
-        <v>0.0383</v>
+        <v>0.0629</v>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>44.2 Days</t>
-        </is>
-      </c>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>OPTIMAL</t>
+          <t>42.0 Days</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>CONTROLLED</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>Onboard &amp; Retain</t>
+          <t>Automate Screening</t>
         </is>
       </c>
     </row>
     <row r="14"/>
     <row r="15"/>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>SOURCING CHANNEL EFFICIENCY &amp; COST-PER-HIRE MATRIX</t>
         </is>
@@ -829,25 +829,25 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Employee Referral</t>
+          <t>Direct Sourcing Outreach</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>9071</v>
+        <v>10960</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>650</v>
+        <v>837</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>0.07165692867379561</v>
-      </c>
-      <c r="E18" s="14" t="n">
-        <v>10885200</v>
-      </c>
-      <c r="F18" s="14" t="n">
-        <v>16746.46153846154</v>
-      </c>
-      <c r="G18" s="12" t="inlineStr">
+        <v>0.07636861313868613</v>
+      </c>
+      <c r="E18" s="13" t="n">
+        <v>9328178.289999954</v>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>11144.7769295101</v>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
         <is>
           <t>HIGH ROI (EXPAND BUDGET)</t>
         </is>
@@ -856,25 +856,25 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>LinkedIn Recruiter</t>
+          <t>Employee Referral</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
-        <v>18886</v>
+        <v>7466</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>493</v>
+        <v>574</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>0.02610399237530446</v>
-      </c>
-      <c r="E19" s="14" t="n">
-        <v>8498700</v>
-      </c>
-      <c r="F19" s="14" t="n">
-        <v>17238.74239350913</v>
-      </c>
-      <c r="G19" s="12" t="inlineStr">
+        <v>0.07688186445218323</v>
+      </c>
+      <c r="E19" s="13" t="n">
+        <v>13433426.36999996</v>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>23403.18182926823</v>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
         <is>
           <t>HIGH ROI (EXPAND BUDGET)</t>
         </is>
@@ -883,25 +883,25 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Inbound Careers Portal</t>
+          <t>LinkedIn Jobs</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>12019</v>
+        <v>19045</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>308</v>
+        <v>405</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>0.0256260920209668</v>
-      </c>
-      <c r="E20" s="14" t="n">
-        <v>600950</v>
-      </c>
-      <c r="F20" s="14" t="n">
-        <v>1951.136363636364</v>
-      </c>
-      <c r="G20" s="12" t="inlineStr">
+        <v>0.02126542399579942</v>
+      </c>
+      <c r="E20" s="13" t="n">
+        <v>6664119.390000041</v>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>16454.61577777788</v>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
         <is>
           <t>HIGH ROI (EXPAND BUDGET)</t>
         </is>
@@ -910,54 +910,54 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Direct Sourcing Outreach</t>
+          <t>External Headhunting Agency</t>
         </is>
       </c>
       <c r="B21" s="7" t="n">
-        <v>4102</v>
+        <v>4999</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>301</v>
+        <v>381</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>0.07337883959044368</v>
-      </c>
-      <c r="E21" s="14" t="n">
-        <v>1148560</v>
-      </c>
-      <c r="F21" s="14" t="n">
-        <v>3815.813953488372</v>
-      </c>
-      <c r="G21" s="12" t="inlineStr">
-        <is>
-          <t>HIGH ROI (EXPAND BUDGET)</t>
+        <v>0.07621524304860972</v>
+      </c>
+      <c r="E21" s="13" t="n">
+        <v>57346190.24999982</v>
+      </c>
+      <c r="F21" s="13" t="n">
+        <v>150514.9350393696</v>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>HIGH COST (AUDIT CONTRACT)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>External Headhunting Agency</t>
+          <t>Inbound Careers Page</t>
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>5922</v>
+        <v>7530</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>0.02769334684228301</v>
-      </c>
-      <c r="E22" s="14" t="n">
-        <v>32571000</v>
-      </c>
-      <c r="F22" s="14" t="n">
-        <v>198603.6585365854</v>
-      </c>
-      <c r="G22" s="15" t="inlineStr">
-        <is>
-          <t>HIGH COST (AUDIT CONTRACT)</t>
+        <v>0.02390438247011952</v>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>339480.1999999998</v>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>1886.00111111111</v>
+      </c>
+      <c r="G22" s="14" t="inlineStr">
+        <is>
+          <t>HIGH ROI (EXPAND BUDGET)</t>
         </is>
       </c>
     </row>

</xml_diff>